<commit_message>
feat(booking): add no_hp column to participants and update excel template download
</commit_message>
<xml_diff>
--- a/template_peserta_baru_kosong.xlsx
+++ b/template_peserta_baru_kosong.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Peserta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Peserta" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,13 +502,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -521,7 +522,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Catatan: Jangan mengubah nama header di baris 4. Isi Kolom D hanya dengan 'L' atau 'P'.</t>
+          <t>Catatan: Jangan mengubah nama header di baris 4. Kolom D (No HP) wajib diisi angka. Kolom E hanya 'L' atau 'P'.</t>
         </is>
       </c>
     </row>
@@ -543,6 +544,11 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>No HP</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>Jenis Kelamin</t>
         </is>
       </c>
@@ -551,96 +557,76 @@
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="6" t="inlineStr"/>
       <c r="B6" s="6" t="inlineStr"/>
       <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr"/>
       <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="6" t="inlineStr"/>
       <c r="B8" s="6" t="inlineStr"/>
       <c r="C8" s="6" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="6" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr"/>
       <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="6" t="inlineStr"/>
       <c r="B12" s="6" t="inlineStr"/>
       <c r="C12" s="6" t="inlineStr"/>
-      <c r="D12" s="7" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="6" t="inlineStr"/>
       <c r="B14" s="6" t="inlineStr"/>
       <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr"/>
-      <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="6" t="inlineStr"/>
-      <c r="B18" s="6" t="inlineStr"/>
-      <c r="C18" s="6" t="inlineStr"/>
-      <c r="D18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>